<commit_message>
Fix conditional-format fill color (dxf bgColor) and widen day columns
Conditional formatting fills were written with fgColor only; Excel reads
bgColor for solid dxf fills, so no color (even weekend shading) appeared.
Set both fg/bg colors. Also widen calendar day columns so date numbers
are not cramped.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014KwWVchh41MC44Bg6BEHQP
</commit_message>
<xml_diff>
--- a/スケジュール_365日.xlsx
+++ b/スケジュール_365日.xlsx
@@ -70,21 +70,25 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002E5395"/>
+        <bgColor rgb="002E5395"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="005BA72B"/>
+        <bgColor rgb="005BA72B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00404040"/>
+        <bgColor rgb="00404040"/>
       </patternFill>
     </fill>
   </fills>
@@ -164,6 +168,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="002E5395"/>
+          <bgColor rgb="002E5395"/>
         </patternFill>
       </fill>
     </dxf>
@@ -171,6 +176,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="005BA72B"/>
+          <bgColor rgb="005BA72B"/>
         </patternFill>
       </fill>
     </dxf>
@@ -178,6 +184,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00E4E7F0"/>
+          <bgColor rgb="00E4E7F0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -553,371 +560,371 @@
     <col width="9" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="5" customWidth="1" min="7" max="7"/>
-    <col width="2.6" customWidth="1" min="8" max="8"/>
-    <col width="2.6" customWidth="1" min="9" max="9"/>
-    <col width="2.6" customWidth="1" min="10" max="10"/>
-    <col width="2.6" customWidth="1" min="11" max="11"/>
-    <col width="2.6" customWidth="1" min="12" max="12"/>
-    <col width="2.6" customWidth="1" min="13" max="13"/>
-    <col width="2.6" customWidth="1" min="14" max="14"/>
-    <col width="2.6" customWidth="1" min="15" max="15"/>
-    <col width="2.6" customWidth="1" min="16" max="16"/>
-    <col width="2.6" customWidth="1" min="17" max="17"/>
-    <col width="2.6" customWidth="1" min="18" max="18"/>
-    <col width="2.6" customWidth="1" min="19" max="19"/>
-    <col width="2.6" customWidth="1" min="20" max="20"/>
-    <col width="2.6" customWidth="1" min="21" max="21"/>
-    <col width="2.6" customWidth="1" min="22" max="22"/>
-    <col width="2.6" customWidth="1" min="23" max="23"/>
-    <col width="2.6" customWidth="1" min="24" max="24"/>
-    <col width="2.6" customWidth="1" min="25" max="25"/>
-    <col width="2.6" customWidth="1" min="26" max="26"/>
-    <col width="2.6" customWidth="1" min="27" max="27"/>
-    <col width="2.6" customWidth="1" min="28" max="28"/>
-    <col width="2.6" customWidth="1" min="29" max="29"/>
-    <col width="2.6" customWidth="1" min="30" max="30"/>
-    <col width="2.6" customWidth="1" min="31" max="31"/>
-    <col width="2.6" customWidth="1" min="32" max="32"/>
-    <col width="2.6" customWidth="1" min="33" max="33"/>
-    <col width="2.6" customWidth="1" min="34" max="34"/>
-    <col width="2.6" customWidth="1" min="35" max="35"/>
-    <col width="2.6" customWidth="1" min="36" max="36"/>
-    <col width="2.6" customWidth="1" min="37" max="37"/>
-    <col width="2.6" customWidth="1" min="38" max="38"/>
-    <col width="2.6" customWidth="1" min="39" max="39"/>
-    <col width="2.6" customWidth="1" min="40" max="40"/>
-    <col width="2.6" customWidth="1" min="41" max="41"/>
-    <col width="2.6" customWidth="1" min="42" max="42"/>
-    <col width="2.6" customWidth="1" min="43" max="43"/>
-    <col width="2.6" customWidth="1" min="44" max="44"/>
-    <col width="2.6" customWidth="1" min="45" max="45"/>
-    <col width="2.6" customWidth="1" min="46" max="46"/>
-    <col width="2.6" customWidth="1" min="47" max="47"/>
-    <col width="2.6" customWidth="1" min="48" max="48"/>
-    <col width="2.6" customWidth="1" min="49" max="49"/>
-    <col width="2.6" customWidth="1" min="50" max="50"/>
-    <col width="2.6" customWidth="1" min="51" max="51"/>
-    <col width="2.6" customWidth="1" min="52" max="52"/>
-    <col width="2.6" customWidth="1" min="53" max="53"/>
-    <col width="2.6" customWidth="1" min="54" max="54"/>
-    <col width="2.6" customWidth="1" min="55" max="55"/>
-    <col width="2.6" customWidth="1" min="56" max="56"/>
-    <col width="2.6" customWidth="1" min="57" max="57"/>
-    <col width="2.6" customWidth="1" min="58" max="58"/>
-    <col width="2.6" customWidth="1" min="59" max="59"/>
-    <col width="2.6" customWidth="1" min="60" max="60"/>
-    <col width="2.6" customWidth="1" min="61" max="61"/>
-    <col width="2.6" customWidth="1" min="62" max="62"/>
-    <col width="2.6" customWidth="1" min="63" max="63"/>
-    <col width="2.6" customWidth="1" min="64" max="64"/>
-    <col width="2.6" customWidth="1" min="65" max="65"/>
-    <col width="2.6" customWidth="1" min="66" max="66"/>
-    <col width="2.6" customWidth="1" min="67" max="67"/>
-    <col width="2.6" customWidth="1" min="68" max="68"/>
-    <col width="2.6" customWidth="1" min="69" max="69"/>
-    <col width="2.6" customWidth="1" min="70" max="70"/>
-    <col width="2.6" customWidth="1" min="71" max="71"/>
-    <col width="2.6" customWidth="1" min="72" max="72"/>
-    <col width="2.6" customWidth="1" min="73" max="73"/>
-    <col width="2.6" customWidth="1" min="74" max="74"/>
-    <col width="2.6" customWidth="1" min="75" max="75"/>
-    <col width="2.6" customWidth="1" min="76" max="76"/>
-    <col width="2.6" customWidth="1" min="77" max="77"/>
-    <col width="2.6" customWidth="1" min="78" max="78"/>
-    <col width="2.6" customWidth="1" min="79" max="79"/>
-    <col width="2.6" customWidth="1" min="80" max="80"/>
-    <col width="2.6" customWidth="1" min="81" max="81"/>
-    <col width="2.6" customWidth="1" min="82" max="82"/>
-    <col width="2.6" customWidth="1" min="83" max="83"/>
-    <col width="2.6" customWidth="1" min="84" max="84"/>
-    <col width="2.6" customWidth="1" min="85" max="85"/>
-    <col width="2.6" customWidth="1" min="86" max="86"/>
-    <col width="2.6" customWidth="1" min="87" max="87"/>
-    <col width="2.6" customWidth="1" min="88" max="88"/>
-    <col width="2.6" customWidth="1" min="89" max="89"/>
-    <col width="2.6" customWidth="1" min="90" max="90"/>
-    <col width="2.6" customWidth="1" min="91" max="91"/>
-    <col width="2.6" customWidth="1" min="92" max="92"/>
-    <col width="2.6" customWidth="1" min="93" max="93"/>
-    <col width="2.6" customWidth="1" min="94" max="94"/>
-    <col width="2.6" customWidth="1" min="95" max="95"/>
-    <col width="2.6" customWidth="1" min="96" max="96"/>
-    <col width="2.6" customWidth="1" min="97" max="97"/>
-    <col width="2.6" customWidth="1" min="98" max="98"/>
-    <col width="2.6" customWidth="1" min="99" max="99"/>
-    <col width="2.6" customWidth="1" min="100" max="100"/>
-    <col width="2.6" customWidth="1" min="101" max="101"/>
-    <col width="2.6" customWidth="1" min="102" max="102"/>
-    <col width="2.6" customWidth="1" min="103" max="103"/>
-    <col width="2.6" customWidth="1" min="104" max="104"/>
-    <col width="2.6" customWidth="1" min="105" max="105"/>
-    <col width="2.6" customWidth="1" min="106" max="106"/>
-    <col width="2.6" customWidth="1" min="107" max="107"/>
-    <col width="2.6" customWidth="1" min="108" max="108"/>
-    <col width="2.6" customWidth="1" min="109" max="109"/>
-    <col width="2.6" customWidth="1" min="110" max="110"/>
-    <col width="2.6" customWidth="1" min="111" max="111"/>
-    <col width="2.6" customWidth="1" min="112" max="112"/>
-    <col width="2.6" customWidth="1" min="113" max="113"/>
-    <col width="2.6" customWidth="1" min="114" max="114"/>
-    <col width="2.6" customWidth="1" min="115" max="115"/>
-    <col width="2.6" customWidth="1" min="116" max="116"/>
-    <col width="2.6" customWidth="1" min="117" max="117"/>
-    <col width="2.6" customWidth="1" min="118" max="118"/>
-    <col width="2.6" customWidth="1" min="119" max="119"/>
-    <col width="2.6" customWidth="1" min="120" max="120"/>
-    <col width="2.6" customWidth="1" min="121" max="121"/>
-    <col width="2.6" customWidth="1" min="122" max="122"/>
-    <col width="2.6" customWidth="1" min="123" max="123"/>
-    <col width="2.6" customWidth="1" min="124" max="124"/>
-    <col width="2.6" customWidth="1" min="125" max="125"/>
-    <col width="2.6" customWidth="1" min="126" max="126"/>
-    <col width="2.6" customWidth="1" min="127" max="127"/>
-    <col width="2.6" customWidth="1" min="128" max="128"/>
-    <col width="2.6" customWidth="1" min="129" max="129"/>
-    <col width="2.6" customWidth="1" min="130" max="130"/>
-    <col width="2.6" customWidth="1" min="131" max="131"/>
-    <col width="2.6" customWidth="1" min="132" max="132"/>
-    <col width="2.6" customWidth="1" min="133" max="133"/>
-    <col width="2.6" customWidth="1" min="134" max="134"/>
-    <col width="2.6" customWidth="1" min="135" max="135"/>
-    <col width="2.6" customWidth="1" min="136" max="136"/>
-    <col width="2.6" customWidth="1" min="137" max="137"/>
-    <col width="2.6" customWidth="1" min="138" max="138"/>
-    <col width="2.6" customWidth="1" min="139" max="139"/>
-    <col width="2.6" customWidth="1" min="140" max="140"/>
-    <col width="2.6" customWidth="1" min="141" max="141"/>
-    <col width="2.6" customWidth="1" min="142" max="142"/>
-    <col width="2.6" customWidth="1" min="143" max="143"/>
-    <col width="2.6" customWidth="1" min="144" max="144"/>
-    <col width="2.6" customWidth="1" min="145" max="145"/>
-    <col width="2.6" customWidth="1" min="146" max="146"/>
-    <col width="2.6" customWidth="1" min="147" max="147"/>
-    <col width="2.6" customWidth="1" min="148" max="148"/>
-    <col width="2.6" customWidth="1" min="149" max="149"/>
-    <col width="2.6" customWidth="1" min="150" max="150"/>
-    <col width="2.6" customWidth="1" min="151" max="151"/>
-    <col width="2.6" customWidth="1" min="152" max="152"/>
-    <col width="2.6" customWidth="1" min="153" max="153"/>
-    <col width="2.6" customWidth="1" min="154" max="154"/>
-    <col width="2.6" customWidth="1" min="155" max="155"/>
-    <col width="2.6" customWidth="1" min="156" max="156"/>
-    <col width="2.6" customWidth="1" min="157" max="157"/>
-    <col width="2.6" customWidth="1" min="158" max="158"/>
-    <col width="2.6" customWidth="1" min="159" max="159"/>
-    <col width="2.6" customWidth="1" min="160" max="160"/>
-    <col width="2.6" customWidth="1" min="161" max="161"/>
-    <col width="2.6" customWidth="1" min="162" max="162"/>
-    <col width="2.6" customWidth="1" min="163" max="163"/>
-    <col width="2.6" customWidth="1" min="164" max="164"/>
-    <col width="2.6" customWidth="1" min="165" max="165"/>
-    <col width="2.6" customWidth="1" min="166" max="166"/>
-    <col width="2.6" customWidth="1" min="167" max="167"/>
-    <col width="2.6" customWidth="1" min="168" max="168"/>
-    <col width="2.6" customWidth="1" min="169" max="169"/>
-    <col width="2.6" customWidth="1" min="170" max="170"/>
-    <col width="2.6" customWidth="1" min="171" max="171"/>
-    <col width="2.6" customWidth="1" min="172" max="172"/>
-    <col width="2.6" customWidth="1" min="173" max="173"/>
-    <col width="2.6" customWidth="1" min="174" max="174"/>
-    <col width="2.6" customWidth="1" min="175" max="175"/>
-    <col width="2.6" customWidth="1" min="176" max="176"/>
-    <col width="2.6" customWidth="1" min="177" max="177"/>
-    <col width="2.6" customWidth="1" min="178" max="178"/>
-    <col width="2.6" customWidth="1" min="179" max="179"/>
-    <col width="2.6" customWidth="1" min="180" max="180"/>
-    <col width="2.6" customWidth="1" min="181" max="181"/>
-    <col width="2.6" customWidth="1" min="182" max="182"/>
-    <col width="2.6" customWidth="1" min="183" max="183"/>
-    <col width="2.6" customWidth="1" min="184" max="184"/>
-    <col width="2.6" customWidth="1" min="185" max="185"/>
-    <col width="2.6" customWidth="1" min="186" max="186"/>
-    <col width="2.6" customWidth="1" min="187" max="187"/>
-    <col width="2.6" customWidth="1" min="188" max="188"/>
-    <col width="2.6" customWidth="1" min="189" max="189"/>
-    <col width="2.6" customWidth="1" min="190" max="190"/>
-    <col width="2.6" customWidth="1" min="191" max="191"/>
-    <col width="2.6" customWidth="1" min="192" max="192"/>
-    <col width="2.6" customWidth="1" min="193" max="193"/>
-    <col width="2.6" customWidth="1" min="194" max="194"/>
-    <col width="2.6" customWidth="1" min="195" max="195"/>
-    <col width="2.6" customWidth="1" min="196" max="196"/>
-    <col width="2.6" customWidth="1" min="197" max="197"/>
-    <col width="2.6" customWidth="1" min="198" max="198"/>
-    <col width="2.6" customWidth="1" min="199" max="199"/>
-    <col width="2.6" customWidth="1" min="200" max="200"/>
-    <col width="2.6" customWidth="1" min="201" max="201"/>
-    <col width="2.6" customWidth="1" min="202" max="202"/>
-    <col width="2.6" customWidth="1" min="203" max="203"/>
-    <col width="2.6" customWidth="1" min="204" max="204"/>
-    <col width="2.6" customWidth="1" min="205" max="205"/>
-    <col width="2.6" customWidth="1" min="206" max="206"/>
-    <col width="2.6" customWidth="1" min="207" max="207"/>
-    <col width="2.6" customWidth="1" min="208" max="208"/>
-    <col width="2.6" customWidth="1" min="209" max="209"/>
-    <col width="2.6" customWidth="1" min="210" max="210"/>
-    <col width="2.6" customWidth="1" min="211" max="211"/>
-    <col width="2.6" customWidth="1" min="212" max="212"/>
-    <col width="2.6" customWidth="1" min="213" max="213"/>
-    <col width="2.6" customWidth="1" min="214" max="214"/>
-    <col width="2.6" customWidth="1" min="215" max="215"/>
-    <col width="2.6" customWidth="1" min="216" max="216"/>
-    <col width="2.6" customWidth="1" min="217" max="217"/>
-    <col width="2.6" customWidth="1" min="218" max="218"/>
-    <col width="2.6" customWidth="1" min="219" max="219"/>
-    <col width="2.6" customWidth="1" min="220" max="220"/>
-    <col width="2.6" customWidth="1" min="221" max="221"/>
-    <col width="2.6" customWidth="1" min="222" max="222"/>
-    <col width="2.6" customWidth="1" min="223" max="223"/>
-    <col width="2.6" customWidth="1" min="224" max="224"/>
-    <col width="2.6" customWidth="1" min="225" max="225"/>
-    <col width="2.6" customWidth="1" min="226" max="226"/>
-    <col width="2.6" customWidth="1" min="227" max="227"/>
-    <col width="2.6" customWidth="1" min="228" max="228"/>
-    <col width="2.6" customWidth="1" min="229" max="229"/>
-    <col width="2.6" customWidth="1" min="230" max="230"/>
-    <col width="2.6" customWidth="1" min="231" max="231"/>
-    <col width="2.6" customWidth="1" min="232" max="232"/>
-    <col width="2.6" customWidth="1" min="233" max="233"/>
-    <col width="2.6" customWidth="1" min="234" max="234"/>
-    <col width="2.6" customWidth="1" min="235" max="235"/>
-    <col width="2.6" customWidth="1" min="236" max="236"/>
-    <col width="2.6" customWidth="1" min="237" max="237"/>
-    <col width="2.6" customWidth="1" min="238" max="238"/>
-    <col width="2.6" customWidth="1" min="239" max="239"/>
-    <col width="2.6" customWidth="1" min="240" max="240"/>
-    <col width="2.6" customWidth="1" min="241" max="241"/>
-    <col width="2.6" customWidth="1" min="242" max="242"/>
-    <col width="2.6" customWidth="1" min="243" max="243"/>
-    <col width="2.6" customWidth="1" min="244" max="244"/>
-    <col width="2.6" customWidth="1" min="245" max="245"/>
-    <col width="2.6" customWidth="1" min="246" max="246"/>
-    <col width="2.6" customWidth="1" min="247" max="247"/>
-    <col width="2.6" customWidth="1" min="248" max="248"/>
-    <col width="2.6" customWidth="1" min="249" max="249"/>
-    <col width="2.6" customWidth="1" min="250" max="250"/>
-    <col width="2.6" customWidth="1" min="251" max="251"/>
-    <col width="2.6" customWidth="1" min="252" max="252"/>
-    <col width="2.6" customWidth="1" min="253" max="253"/>
-    <col width="2.6" customWidth="1" min="254" max="254"/>
-    <col width="2.6" customWidth="1" min="255" max="255"/>
-    <col width="2.6" customWidth="1" min="256" max="256"/>
-    <col width="2.6" customWidth="1" min="257" max="257"/>
-    <col width="2.6" customWidth="1" min="258" max="258"/>
-    <col width="2.6" customWidth="1" min="259" max="259"/>
-    <col width="2.6" customWidth="1" min="260" max="260"/>
-    <col width="2.6" customWidth="1" min="261" max="261"/>
-    <col width="2.6" customWidth="1" min="262" max="262"/>
-    <col width="2.6" customWidth="1" min="263" max="263"/>
-    <col width="2.6" customWidth="1" min="264" max="264"/>
-    <col width="2.6" customWidth="1" min="265" max="265"/>
-    <col width="2.6" customWidth="1" min="266" max="266"/>
-    <col width="2.6" customWidth="1" min="267" max="267"/>
-    <col width="2.6" customWidth="1" min="268" max="268"/>
-    <col width="2.6" customWidth="1" min="269" max="269"/>
-    <col width="2.6" customWidth="1" min="270" max="270"/>
-    <col width="2.6" customWidth="1" min="271" max="271"/>
-    <col width="2.6" customWidth="1" min="272" max="272"/>
-    <col width="2.6" customWidth="1" min="273" max="273"/>
-    <col width="2.6" customWidth="1" min="274" max="274"/>
-    <col width="2.6" customWidth="1" min="275" max="275"/>
-    <col width="2.6" customWidth="1" min="276" max="276"/>
-    <col width="2.6" customWidth="1" min="277" max="277"/>
-    <col width="2.6" customWidth="1" min="278" max="278"/>
-    <col width="2.6" customWidth="1" min="279" max="279"/>
-    <col width="2.6" customWidth="1" min="280" max="280"/>
-    <col width="2.6" customWidth="1" min="281" max="281"/>
-    <col width="2.6" customWidth="1" min="282" max="282"/>
-    <col width="2.6" customWidth="1" min="283" max="283"/>
-    <col width="2.6" customWidth="1" min="284" max="284"/>
-    <col width="2.6" customWidth="1" min="285" max="285"/>
-    <col width="2.6" customWidth="1" min="286" max="286"/>
-    <col width="2.6" customWidth="1" min="287" max="287"/>
-    <col width="2.6" customWidth="1" min="288" max="288"/>
-    <col width="2.6" customWidth="1" min="289" max="289"/>
-    <col width="2.6" customWidth="1" min="290" max="290"/>
-    <col width="2.6" customWidth="1" min="291" max="291"/>
-    <col width="2.6" customWidth="1" min="292" max="292"/>
-    <col width="2.6" customWidth="1" min="293" max="293"/>
-    <col width="2.6" customWidth="1" min="294" max="294"/>
-    <col width="2.6" customWidth="1" min="295" max="295"/>
-    <col width="2.6" customWidth="1" min="296" max="296"/>
-    <col width="2.6" customWidth="1" min="297" max="297"/>
-    <col width="2.6" customWidth="1" min="298" max="298"/>
-    <col width="2.6" customWidth="1" min="299" max="299"/>
-    <col width="2.6" customWidth="1" min="300" max="300"/>
-    <col width="2.6" customWidth="1" min="301" max="301"/>
-    <col width="2.6" customWidth="1" min="302" max="302"/>
-    <col width="2.6" customWidth="1" min="303" max="303"/>
-    <col width="2.6" customWidth="1" min="304" max="304"/>
-    <col width="2.6" customWidth="1" min="305" max="305"/>
-    <col width="2.6" customWidth="1" min="306" max="306"/>
-    <col width="2.6" customWidth="1" min="307" max="307"/>
-    <col width="2.6" customWidth="1" min="308" max="308"/>
-    <col width="2.6" customWidth="1" min="309" max="309"/>
-    <col width="2.6" customWidth="1" min="310" max="310"/>
-    <col width="2.6" customWidth="1" min="311" max="311"/>
-    <col width="2.6" customWidth="1" min="312" max="312"/>
-    <col width="2.6" customWidth="1" min="313" max="313"/>
-    <col width="2.6" customWidth="1" min="314" max="314"/>
-    <col width="2.6" customWidth="1" min="315" max="315"/>
-    <col width="2.6" customWidth="1" min="316" max="316"/>
-    <col width="2.6" customWidth="1" min="317" max="317"/>
-    <col width="2.6" customWidth="1" min="318" max="318"/>
-    <col width="2.6" customWidth="1" min="319" max="319"/>
-    <col width="2.6" customWidth="1" min="320" max="320"/>
-    <col width="2.6" customWidth="1" min="321" max="321"/>
-    <col width="2.6" customWidth="1" min="322" max="322"/>
-    <col width="2.6" customWidth="1" min="323" max="323"/>
-    <col width="2.6" customWidth="1" min="324" max="324"/>
-    <col width="2.6" customWidth="1" min="325" max="325"/>
-    <col width="2.6" customWidth="1" min="326" max="326"/>
-    <col width="2.6" customWidth="1" min="327" max="327"/>
-    <col width="2.6" customWidth="1" min="328" max="328"/>
-    <col width="2.6" customWidth="1" min="329" max="329"/>
-    <col width="2.6" customWidth="1" min="330" max="330"/>
-    <col width="2.6" customWidth="1" min="331" max="331"/>
-    <col width="2.6" customWidth="1" min="332" max="332"/>
-    <col width="2.6" customWidth="1" min="333" max="333"/>
-    <col width="2.6" customWidth="1" min="334" max="334"/>
-    <col width="2.6" customWidth="1" min="335" max="335"/>
-    <col width="2.6" customWidth="1" min="336" max="336"/>
-    <col width="2.6" customWidth="1" min="337" max="337"/>
-    <col width="2.6" customWidth="1" min="338" max="338"/>
-    <col width="2.6" customWidth="1" min="339" max="339"/>
-    <col width="2.6" customWidth="1" min="340" max="340"/>
-    <col width="2.6" customWidth="1" min="341" max="341"/>
-    <col width="2.6" customWidth="1" min="342" max="342"/>
-    <col width="2.6" customWidth="1" min="343" max="343"/>
-    <col width="2.6" customWidth="1" min="344" max="344"/>
-    <col width="2.6" customWidth="1" min="345" max="345"/>
-    <col width="2.6" customWidth="1" min="346" max="346"/>
-    <col width="2.6" customWidth="1" min="347" max="347"/>
-    <col width="2.6" customWidth="1" min="348" max="348"/>
-    <col width="2.6" customWidth="1" min="349" max="349"/>
-    <col width="2.6" customWidth="1" min="350" max="350"/>
-    <col width="2.6" customWidth="1" min="351" max="351"/>
-    <col width="2.6" customWidth="1" min="352" max="352"/>
-    <col width="2.6" customWidth="1" min="353" max="353"/>
-    <col width="2.6" customWidth="1" min="354" max="354"/>
-    <col width="2.6" customWidth="1" min="355" max="355"/>
-    <col width="2.6" customWidth="1" min="356" max="356"/>
-    <col width="2.6" customWidth="1" min="357" max="357"/>
-    <col width="2.6" customWidth="1" min="358" max="358"/>
-    <col width="2.6" customWidth="1" min="359" max="359"/>
-    <col width="2.6" customWidth="1" min="360" max="360"/>
-    <col width="2.6" customWidth="1" min="361" max="361"/>
-    <col width="2.6" customWidth="1" min="362" max="362"/>
-    <col width="2.6" customWidth="1" min="363" max="363"/>
-    <col width="2.6" customWidth="1" min="364" max="364"/>
-    <col width="2.6" customWidth="1" min="365" max="365"/>
-    <col width="2.6" customWidth="1" min="366" max="366"/>
-    <col width="2.6" customWidth="1" min="367" max="367"/>
-    <col width="2.6" customWidth="1" min="368" max="368"/>
-    <col width="2.6" customWidth="1" min="369" max="369"/>
-    <col width="2.6" customWidth="1" min="370" max="370"/>
-    <col width="2.6" customWidth="1" min="371" max="371"/>
-    <col width="2.6" customWidth="1" min="372" max="372"/>
+    <col width="3.4" customWidth="1" min="8" max="8"/>
+    <col width="3.4" customWidth="1" min="9" max="9"/>
+    <col width="3.4" customWidth="1" min="10" max="10"/>
+    <col width="3.4" customWidth="1" min="11" max="11"/>
+    <col width="3.4" customWidth="1" min="12" max="12"/>
+    <col width="3.4" customWidth="1" min="13" max="13"/>
+    <col width="3.4" customWidth="1" min="14" max="14"/>
+    <col width="3.4" customWidth="1" min="15" max="15"/>
+    <col width="3.4" customWidth="1" min="16" max="16"/>
+    <col width="3.4" customWidth="1" min="17" max="17"/>
+    <col width="3.4" customWidth="1" min="18" max="18"/>
+    <col width="3.4" customWidth="1" min="19" max="19"/>
+    <col width="3.4" customWidth="1" min="20" max="20"/>
+    <col width="3.4" customWidth="1" min="21" max="21"/>
+    <col width="3.4" customWidth="1" min="22" max="22"/>
+    <col width="3.4" customWidth="1" min="23" max="23"/>
+    <col width="3.4" customWidth="1" min="24" max="24"/>
+    <col width="3.4" customWidth="1" min="25" max="25"/>
+    <col width="3.4" customWidth="1" min="26" max="26"/>
+    <col width="3.4" customWidth="1" min="27" max="27"/>
+    <col width="3.4" customWidth="1" min="28" max="28"/>
+    <col width="3.4" customWidth="1" min="29" max="29"/>
+    <col width="3.4" customWidth="1" min="30" max="30"/>
+    <col width="3.4" customWidth="1" min="31" max="31"/>
+    <col width="3.4" customWidth="1" min="32" max="32"/>
+    <col width="3.4" customWidth="1" min="33" max="33"/>
+    <col width="3.4" customWidth="1" min="34" max="34"/>
+    <col width="3.4" customWidth="1" min="35" max="35"/>
+    <col width="3.4" customWidth="1" min="36" max="36"/>
+    <col width="3.4" customWidth="1" min="37" max="37"/>
+    <col width="3.4" customWidth="1" min="38" max="38"/>
+    <col width="3.4" customWidth="1" min="39" max="39"/>
+    <col width="3.4" customWidth="1" min="40" max="40"/>
+    <col width="3.4" customWidth="1" min="41" max="41"/>
+    <col width="3.4" customWidth="1" min="42" max="42"/>
+    <col width="3.4" customWidth="1" min="43" max="43"/>
+    <col width="3.4" customWidth="1" min="44" max="44"/>
+    <col width="3.4" customWidth="1" min="45" max="45"/>
+    <col width="3.4" customWidth="1" min="46" max="46"/>
+    <col width="3.4" customWidth="1" min="47" max="47"/>
+    <col width="3.4" customWidth="1" min="48" max="48"/>
+    <col width="3.4" customWidth="1" min="49" max="49"/>
+    <col width="3.4" customWidth="1" min="50" max="50"/>
+    <col width="3.4" customWidth="1" min="51" max="51"/>
+    <col width="3.4" customWidth="1" min="52" max="52"/>
+    <col width="3.4" customWidth="1" min="53" max="53"/>
+    <col width="3.4" customWidth="1" min="54" max="54"/>
+    <col width="3.4" customWidth="1" min="55" max="55"/>
+    <col width="3.4" customWidth="1" min="56" max="56"/>
+    <col width="3.4" customWidth="1" min="57" max="57"/>
+    <col width="3.4" customWidth="1" min="58" max="58"/>
+    <col width="3.4" customWidth="1" min="59" max="59"/>
+    <col width="3.4" customWidth="1" min="60" max="60"/>
+    <col width="3.4" customWidth="1" min="61" max="61"/>
+    <col width="3.4" customWidth="1" min="62" max="62"/>
+    <col width="3.4" customWidth="1" min="63" max="63"/>
+    <col width="3.4" customWidth="1" min="64" max="64"/>
+    <col width="3.4" customWidth="1" min="65" max="65"/>
+    <col width="3.4" customWidth="1" min="66" max="66"/>
+    <col width="3.4" customWidth="1" min="67" max="67"/>
+    <col width="3.4" customWidth="1" min="68" max="68"/>
+    <col width="3.4" customWidth="1" min="69" max="69"/>
+    <col width="3.4" customWidth="1" min="70" max="70"/>
+    <col width="3.4" customWidth="1" min="71" max="71"/>
+    <col width="3.4" customWidth="1" min="72" max="72"/>
+    <col width="3.4" customWidth="1" min="73" max="73"/>
+    <col width="3.4" customWidth="1" min="74" max="74"/>
+    <col width="3.4" customWidth="1" min="75" max="75"/>
+    <col width="3.4" customWidth="1" min="76" max="76"/>
+    <col width="3.4" customWidth="1" min="77" max="77"/>
+    <col width="3.4" customWidth="1" min="78" max="78"/>
+    <col width="3.4" customWidth="1" min="79" max="79"/>
+    <col width="3.4" customWidth="1" min="80" max="80"/>
+    <col width="3.4" customWidth="1" min="81" max="81"/>
+    <col width="3.4" customWidth="1" min="82" max="82"/>
+    <col width="3.4" customWidth="1" min="83" max="83"/>
+    <col width="3.4" customWidth="1" min="84" max="84"/>
+    <col width="3.4" customWidth="1" min="85" max="85"/>
+    <col width="3.4" customWidth="1" min="86" max="86"/>
+    <col width="3.4" customWidth="1" min="87" max="87"/>
+    <col width="3.4" customWidth="1" min="88" max="88"/>
+    <col width="3.4" customWidth="1" min="89" max="89"/>
+    <col width="3.4" customWidth="1" min="90" max="90"/>
+    <col width="3.4" customWidth="1" min="91" max="91"/>
+    <col width="3.4" customWidth="1" min="92" max="92"/>
+    <col width="3.4" customWidth="1" min="93" max="93"/>
+    <col width="3.4" customWidth="1" min="94" max="94"/>
+    <col width="3.4" customWidth="1" min="95" max="95"/>
+    <col width="3.4" customWidth="1" min="96" max="96"/>
+    <col width="3.4" customWidth="1" min="97" max="97"/>
+    <col width="3.4" customWidth="1" min="98" max="98"/>
+    <col width="3.4" customWidth="1" min="99" max="99"/>
+    <col width="3.4" customWidth="1" min="100" max="100"/>
+    <col width="3.4" customWidth="1" min="101" max="101"/>
+    <col width="3.4" customWidth="1" min="102" max="102"/>
+    <col width="3.4" customWidth="1" min="103" max="103"/>
+    <col width="3.4" customWidth="1" min="104" max="104"/>
+    <col width="3.4" customWidth="1" min="105" max="105"/>
+    <col width="3.4" customWidth="1" min="106" max="106"/>
+    <col width="3.4" customWidth="1" min="107" max="107"/>
+    <col width="3.4" customWidth="1" min="108" max="108"/>
+    <col width="3.4" customWidth="1" min="109" max="109"/>
+    <col width="3.4" customWidth="1" min="110" max="110"/>
+    <col width="3.4" customWidth="1" min="111" max="111"/>
+    <col width="3.4" customWidth="1" min="112" max="112"/>
+    <col width="3.4" customWidth="1" min="113" max="113"/>
+    <col width="3.4" customWidth="1" min="114" max="114"/>
+    <col width="3.4" customWidth="1" min="115" max="115"/>
+    <col width="3.4" customWidth="1" min="116" max="116"/>
+    <col width="3.4" customWidth="1" min="117" max="117"/>
+    <col width="3.4" customWidth="1" min="118" max="118"/>
+    <col width="3.4" customWidth="1" min="119" max="119"/>
+    <col width="3.4" customWidth="1" min="120" max="120"/>
+    <col width="3.4" customWidth="1" min="121" max="121"/>
+    <col width="3.4" customWidth="1" min="122" max="122"/>
+    <col width="3.4" customWidth="1" min="123" max="123"/>
+    <col width="3.4" customWidth="1" min="124" max="124"/>
+    <col width="3.4" customWidth="1" min="125" max="125"/>
+    <col width="3.4" customWidth="1" min="126" max="126"/>
+    <col width="3.4" customWidth="1" min="127" max="127"/>
+    <col width="3.4" customWidth="1" min="128" max="128"/>
+    <col width="3.4" customWidth="1" min="129" max="129"/>
+    <col width="3.4" customWidth="1" min="130" max="130"/>
+    <col width="3.4" customWidth="1" min="131" max="131"/>
+    <col width="3.4" customWidth="1" min="132" max="132"/>
+    <col width="3.4" customWidth="1" min="133" max="133"/>
+    <col width="3.4" customWidth="1" min="134" max="134"/>
+    <col width="3.4" customWidth="1" min="135" max="135"/>
+    <col width="3.4" customWidth="1" min="136" max="136"/>
+    <col width="3.4" customWidth="1" min="137" max="137"/>
+    <col width="3.4" customWidth="1" min="138" max="138"/>
+    <col width="3.4" customWidth="1" min="139" max="139"/>
+    <col width="3.4" customWidth="1" min="140" max="140"/>
+    <col width="3.4" customWidth="1" min="141" max="141"/>
+    <col width="3.4" customWidth="1" min="142" max="142"/>
+    <col width="3.4" customWidth="1" min="143" max="143"/>
+    <col width="3.4" customWidth="1" min="144" max="144"/>
+    <col width="3.4" customWidth="1" min="145" max="145"/>
+    <col width="3.4" customWidth="1" min="146" max="146"/>
+    <col width="3.4" customWidth="1" min="147" max="147"/>
+    <col width="3.4" customWidth="1" min="148" max="148"/>
+    <col width="3.4" customWidth="1" min="149" max="149"/>
+    <col width="3.4" customWidth="1" min="150" max="150"/>
+    <col width="3.4" customWidth="1" min="151" max="151"/>
+    <col width="3.4" customWidth="1" min="152" max="152"/>
+    <col width="3.4" customWidth="1" min="153" max="153"/>
+    <col width="3.4" customWidth="1" min="154" max="154"/>
+    <col width="3.4" customWidth="1" min="155" max="155"/>
+    <col width="3.4" customWidth="1" min="156" max="156"/>
+    <col width="3.4" customWidth="1" min="157" max="157"/>
+    <col width="3.4" customWidth="1" min="158" max="158"/>
+    <col width="3.4" customWidth="1" min="159" max="159"/>
+    <col width="3.4" customWidth="1" min="160" max="160"/>
+    <col width="3.4" customWidth="1" min="161" max="161"/>
+    <col width="3.4" customWidth="1" min="162" max="162"/>
+    <col width="3.4" customWidth="1" min="163" max="163"/>
+    <col width="3.4" customWidth="1" min="164" max="164"/>
+    <col width="3.4" customWidth="1" min="165" max="165"/>
+    <col width="3.4" customWidth="1" min="166" max="166"/>
+    <col width="3.4" customWidth="1" min="167" max="167"/>
+    <col width="3.4" customWidth="1" min="168" max="168"/>
+    <col width="3.4" customWidth="1" min="169" max="169"/>
+    <col width="3.4" customWidth="1" min="170" max="170"/>
+    <col width="3.4" customWidth="1" min="171" max="171"/>
+    <col width="3.4" customWidth="1" min="172" max="172"/>
+    <col width="3.4" customWidth="1" min="173" max="173"/>
+    <col width="3.4" customWidth="1" min="174" max="174"/>
+    <col width="3.4" customWidth="1" min="175" max="175"/>
+    <col width="3.4" customWidth="1" min="176" max="176"/>
+    <col width="3.4" customWidth="1" min="177" max="177"/>
+    <col width="3.4" customWidth="1" min="178" max="178"/>
+    <col width="3.4" customWidth="1" min="179" max="179"/>
+    <col width="3.4" customWidth="1" min="180" max="180"/>
+    <col width="3.4" customWidth="1" min="181" max="181"/>
+    <col width="3.4" customWidth="1" min="182" max="182"/>
+    <col width="3.4" customWidth="1" min="183" max="183"/>
+    <col width="3.4" customWidth="1" min="184" max="184"/>
+    <col width="3.4" customWidth="1" min="185" max="185"/>
+    <col width="3.4" customWidth="1" min="186" max="186"/>
+    <col width="3.4" customWidth="1" min="187" max="187"/>
+    <col width="3.4" customWidth="1" min="188" max="188"/>
+    <col width="3.4" customWidth="1" min="189" max="189"/>
+    <col width="3.4" customWidth="1" min="190" max="190"/>
+    <col width="3.4" customWidth="1" min="191" max="191"/>
+    <col width="3.4" customWidth="1" min="192" max="192"/>
+    <col width="3.4" customWidth="1" min="193" max="193"/>
+    <col width="3.4" customWidth="1" min="194" max="194"/>
+    <col width="3.4" customWidth="1" min="195" max="195"/>
+    <col width="3.4" customWidth="1" min="196" max="196"/>
+    <col width="3.4" customWidth="1" min="197" max="197"/>
+    <col width="3.4" customWidth="1" min="198" max="198"/>
+    <col width="3.4" customWidth="1" min="199" max="199"/>
+    <col width="3.4" customWidth="1" min="200" max="200"/>
+    <col width="3.4" customWidth="1" min="201" max="201"/>
+    <col width="3.4" customWidth="1" min="202" max="202"/>
+    <col width="3.4" customWidth="1" min="203" max="203"/>
+    <col width="3.4" customWidth="1" min="204" max="204"/>
+    <col width="3.4" customWidth="1" min="205" max="205"/>
+    <col width="3.4" customWidth="1" min="206" max="206"/>
+    <col width="3.4" customWidth="1" min="207" max="207"/>
+    <col width="3.4" customWidth="1" min="208" max="208"/>
+    <col width="3.4" customWidth="1" min="209" max="209"/>
+    <col width="3.4" customWidth="1" min="210" max="210"/>
+    <col width="3.4" customWidth="1" min="211" max="211"/>
+    <col width="3.4" customWidth="1" min="212" max="212"/>
+    <col width="3.4" customWidth="1" min="213" max="213"/>
+    <col width="3.4" customWidth="1" min="214" max="214"/>
+    <col width="3.4" customWidth="1" min="215" max="215"/>
+    <col width="3.4" customWidth="1" min="216" max="216"/>
+    <col width="3.4" customWidth="1" min="217" max="217"/>
+    <col width="3.4" customWidth="1" min="218" max="218"/>
+    <col width="3.4" customWidth="1" min="219" max="219"/>
+    <col width="3.4" customWidth="1" min="220" max="220"/>
+    <col width="3.4" customWidth="1" min="221" max="221"/>
+    <col width="3.4" customWidth="1" min="222" max="222"/>
+    <col width="3.4" customWidth="1" min="223" max="223"/>
+    <col width="3.4" customWidth="1" min="224" max="224"/>
+    <col width="3.4" customWidth="1" min="225" max="225"/>
+    <col width="3.4" customWidth="1" min="226" max="226"/>
+    <col width="3.4" customWidth="1" min="227" max="227"/>
+    <col width="3.4" customWidth="1" min="228" max="228"/>
+    <col width="3.4" customWidth="1" min="229" max="229"/>
+    <col width="3.4" customWidth="1" min="230" max="230"/>
+    <col width="3.4" customWidth="1" min="231" max="231"/>
+    <col width="3.4" customWidth="1" min="232" max="232"/>
+    <col width="3.4" customWidth="1" min="233" max="233"/>
+    <col width="3.4" customWidth="1" min="234" max="234"/>
+    <col width="3.4" customWidth="1" min="235" max="235"/>
+    <col width="3.4" customWidth="1" min="236" max="236"/>
+    <col width="3.4" customWidth="1" min="237" max="237"/>
+    <col width="3.4" customWidth="1" min="238" max="238"/>
+    <col width="3.4" customWidth="1" min="239" max="239"/>
+    <col width="3.4" customWidth="1" min="240" max="240"/>
+    <col width="3.4" customWidth="1" min="241" max="241"/>
+    <col width="3.4" customWidth="1" min="242" max="242"/>
+    <col width="3.4" customWidth="1" min="243" max="243"/>
+    <col width="3.4" customWidth="1" min="244" max="244"/>
+    <col width="3.4" customWidth="1" min="245" max="245"/>
+    <col width="3.4" customWidth="1" min="246" max="246"/>
+    <col width="3.4" customWidth="1" min="247" max="247"/>
+    <col width="3.4" customWidth="1" min="248" max="248"/>
+    <col width="3.4" customWidth="1" min="249" max="249"/>
+    <col width="3.4" customWidth="1" min="250" max="250"/>
+    <col width="3.4" customWidth="1" min="251" max="251"/>
+    <col width="3.4" customWidth="1" min="252" max="252"/>
+    <col width="3.4" customWidth="1" min="253" max="253"/>
+    <col width="3.4" customWidth="1" min="254" max="254"/>
+    <col width="3.4" customWidth="1" min="255" max="255"/>
+    <col width="3.4" customWidth="1" min="256" max="256"/>
+    <col width="3.4" customWidth="1" min="257" max="257"/>
+    <col width="3.4" customWidth="1" min="258" max="258"/>
+    <col width="3.4" customWidth="1" min="259" max="259"/>
+    <col width="3.4" customWidth="1" min="260" max="260"/>
+    <col width="3.4" customWidth="1" min="261" max="261"/>
+    <col width="3.4" customWidth="1" min="262" max="262"/>
+    <col width="3.4" customWidth="1" min="263" max="263"/>
+    <col width="3.4" customWidth="1" min="264" max="264"/>
+    <col width="3.4" customWidth="1" min="265" max="265"/>
+    <col width="3.4" customWidth="1" min="266" max="266"/>
+    <col width="3.4" customWidth="1" min="267" max="267"/>
+    <col width="3.4" customWidth="1" min="268" max="268"/>
+    <col width="3.4" customWidth="1" min="269" max="269"/>
+    <col width="3.4" customWidth="1" min="270" max="270"/>
+    <col width="3.4" customWidth="1" min="271" max="271"/>
+    <col width="3.4" customWidth="1" min="272" max="272"/>
+    <col width="3.4" customWidth="1" min="273" max="273"/>
+    <col width="3.4" customWidth="1" min="274" max="274"/>
+    <col width="3.4" customWidth="1" min="275" max="275"/>
+    <col width="3.4" customWidth="1" min="276" max="276"/>
+    <col width="3.4" customWidth="1" min="277" max="277"/>
+    <col width="3.4" customWidth="1" min="278" max="278"/>
+    <col width="3.4" customWidth="1" min="279" max="279"/>
+    <col width="3.4" customWidth="1" min="280" max="280"/>
+    <col width="3.4" customWidth="1" min="281" max="281"/>
+    <col width="3.4" customWidth="1" min="282" max="282"/>
+    <col width="3.4" customWidth="1" min="283" max="283"/>
+    <col width="3.4" customWidth="1" min="284" max="284"/>
+    <col width="3.4" customWidth="1" min="285" max="285"/>
+    <col width="3.4" customWidth="1" min="286" max="286"/>
+    <col width="3.4" customWidth="1" min="287" max="287"/>
+    <col width="3.4" customWidth="1" min="288" max="288"/>
+    <col width="3.4" customWidth="1" min="289" max="289"/>
+    <col width="3.4" customWidth="1" min="290" max="290"/>
+    <col width="3.4" customWidth="1" min="291" max="291"/>
+    <col width="3.4" customWidth="1" min="292" max="292"/>
+    <col width="3.4" customWidth="1" min="293" max="293"/>
+    <col width="3.4" customWidth="1" min="294" max="294"/>
+    <col width="3.4" customWidth="1" min="295" max="295"/>
+    <col width="3.4" customWidth="1" min="296" max="296"/>
+    <col width="3.4" customWidth="1" min="297" max="297"/>
+    <col width="3.4" customWidth="1" min="298" max="298"/>
+    <col width="3.4" customWidth="1" min="299" max="299"/>
+    <col width="3.4" customWidth="1" min="300" max="300"/>
+    <col width="3.4" customWidth="1" min="301" max="301"/>
+    <col width="3.4" customWidth="1" min="302" max="302"/>
+    <col width="3.4" customWidth="1" min="303" max="303"/>
+    <col width="3.4" customWidth="1" min="304" max="304"/>
+    <col width="3.4" customWidth="1" min="305" max="305"/>
+    <col width="3.4" customWidth="1" min="306" max="306"/>
+    <col width="3.4" customWidth="1" min="307" max="307"/>
+    <col width="3.4" customWidth="1" min="308" max="308"/>
+    <col width="3.4" customWidth="1" min="309" max="309"/>
+    <col width="3.4" customWidth="1" min="310" max="310"/>
+    <col width="3.4" customWidth="1" min="311" max="311"/>
+    <col width="3.4" customWidth="1" min="312" max="312"/>
+    <col width="3.4" customWidth="1" min="313" max="313"/>
+    <col width="3.4" customWidth="1" min="314" max="314"/>
+    <col width="3.4" customWidth="1" min="315" max="315"/>
+    <col width="3.4" customWidth="1" min="316" max="316"/>
+    <col width="3.4" customWidth="1" min="317" max="317"/>
+    <col width="3.4" customWidth="1" min="318" max="318"/>
+    <col width="3.4" customWidth="1" min="319" max="319"/>
+    <col width="3.4" customWidth="1" min="320" max="320"/>
+    <col width="3.4" customWidth="1" min="321" max="321"/>
+    <col width="3.4" customWidth="1" min="322" max="322"/>
+    <col width="3.4" customWidth="1" min="323" max="323"/>
+    <col width="3.4" customWidth="1" min="324" max="324"/>
+    <col width="3.4" customWidth="1" min="325" max="325"/>
+    <col width="3.4" customWidth="1" min="326" max="326"/>
+    <col width="3.4" customWidth="1" min="327" max="327"/>
+    <col width="3.4" customWidth="1" min="328" max="328"/>
+    <col width="3.4" customWidth="1" min="329" max="329"/>
+    <col width="3.4" customWidth="1" min="330" max="330"/>
+    <col width="3.4" customWidth="1" min="331" max="331"/>
+    <col width="3.4" customWidth="1" min="332" max="332"/>
+    <col width="3.4" customWidth="1" min="333" max="333"/>
+    <col width="3.4" customWidth="1" min="334" max="334"/>
+    <col width="3.4" customWidth="1" min="335" max="335"/>
+    <col width="3.4" customWidth="1" min="336" max="336"/>
+    <col width="3.4" customWidth="1" min="337" max="337"/>
+    <col width="3.4" customWidth="1" min="338" max="338"/>
+    <col width="3.4" customWidth="1" min="339" max="339"/>
+    <col width="3.4" customWidth="1" min="340" max="340"/>
+    <col width="3.4" customWidth="1" min="341" max="341"/>
+    <col width="3.4" customWidth="1" min="342" max="342"/>
+    <col width="3.4" customWidth="1" min="343" max="343"/>
+    <col width="3.4" customWidth="1" min="344" max="344"/>
+    <col width="3.4" customWidth="1" min="345" max="345"/>
+    <col width="3.4" customWidth="1" min="346" max="346"/>
+    <col width="3.4" customWidth="1" min="347" max="347"/>
+    <col width="3.4" customWidth="1" min="348" max="348"/>
+    <col width="3.4" customWidth="1" min="349" max="349"/>
+    <col width="3.4" customWidth="1" min="350" max="350"/>
+    <col width="3.4" customWidth="1" min="351" max="351"/>
+    <col width="3.4" customWidth="1" min="352" max="352"/>
+    <col width="3.4" customWidth="1" min="353" max="353"/>
+    <col width="3.4" customWidth="1" min="354" max="354"/>
+    <col width="3.4" customWidth="1" min="355" max="355"/>
+    <col width="3.4" customWidth="1" min="356" max="356"/>
+    <col width="3.4" customWidth="1" min="357" max="357"/>
+    <col width="3.4" customWidth="1" min="358" max="358"/>
+    <col width="3.4" customWidth="1" min="359" max="359"/>
+    <col width="3.4" customWidth="1" min="360" max="360"/>
+    <col width="3.4" customWidth="1" min="361" max="361"/>
+    <col width="3.4" customWidth="1" min="362" max="362"/>
+    <col width="3.4" customWidth="1" min="363" max="363"/>
+    <col width="3.4" customWidth="1" min="364" max="364"/>
+    <col width="3.4" customWidth="1" min="365" max="365"/>
+    <col width="3.4" customWidth="1" min="366" max="366"/>
+    <col width="3.4" customWidth="1" min="367" max="367"/>
+    <col width="3.4" customWidth="1" min="368" max="368"/>
+    <col width="3.4" customWidth="1" min="369" max="369"/>
+    <col width="3.4" customWidth="1" min="370" max="370"/>
+    <col width="3.4" customWidth="1" min="371" max="371"/>
+    <col width="3.4" customWidth="1" min="372" max="372"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Widen 開始日/締切日/完了日 columns so the base date is not truncated
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014KwWVchh41MC44Bg6BEHQP
</commit_message>
<xml_diff>
--- a/スケジュール_365日.xlsx
+++ b/スケジュール_365日.xlsx
@@ -556,9 +556,9 @@
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="5" customWidth="1" min="7" max="7"/>
     <col width="3.4" customWidth="1" min="8" max="8"/>
     <col width="3.4" customWidth="1" min="9" max="9"/>

</xml_diff>